<commit_message>
Migrate 10 additional Cloud Functions v1 to v2 and update Excel tracker
- Refactored createUsers, deleteUsers, isFullMigratedWP, changePasswordWPFB, generateTokenWP, generateTokenZoom, listCards, setPoints, tokens, and getFbToken into functions/assets/js/
- Exported v2 HTTP onRequest and Callable onCall endpoints in functions/index.js
- Updated functions_v1/functions_v1.xlsx setting REFACTORIZED to true for all 10 migrated functions

Co-authored-by: EMTrvillatoro <99835179+EMTrvillatoro@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/functions_v1/functions_v1.xlsx
+++ b/functions_v1/functions_v1.xlsx
@@ -564,7 +564,7 @@
         <v>changePasswordWPFB</v>
       </c>
       <c r="B21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +628,7 @@
         <v>createUsers</v>
       </c>
       <c r="B29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -644,7 +644,7 @@
         <v>deleteUsers</v>
       </c>
       <c r="B31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -732,7 +732,7 @@
         <v>generateTokenWP</v>
       </c>
       <c r="B42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -740,7 +740,7 @@
         <v>generateTokenZoom</v>
       </c>
       <c r="B43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -780,7 +780,7 @@
         <v>getFbToken</v>
       </c>
       <c r="B48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -820,7 +820,7 @@
         <v>isFullMigratedWP</v>
       </c>
       <c r="B53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -836,7 +836,7 @@
         <v>listCards</v>
       </c>
       <c r="B55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -1052,7 +1052,7 @@
         <v>setPoints</v>
       </c>
       <c r="B82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -1068,7 +1068,7 @@
         <v>tokens</v>
       </c>
       <c r="B84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">

</xml_diff>

<commit_message>
Migrate 12 additional Cloud Functions v1 to v2 and update Excel tracker
- Refactored bq_onRequest_getResponseWebhook, bq_onRequest_newsletters, bq_onRequest_newsletters_update, bq_onRun_campaigns, bq_onRun_contacts, bq_onRun_newsletters, bq_onRun_newsletters_update into functions/assets/js/bigquery/queries.js
- Refactored certificadosBatch into functions/assets/js/certificados/certificadosBatch.js
- Refactored changePassword and checkCode into functions/assets/js/user/
- Refactored checkRepresentantive into functions/assets/js/triggers/plans.js
- Refactored clickMeetingToBQ into functions/assets/js/click-meeting/clickMeetingBQ.js
- Registered and exported v2 endpoints in functions/index.js
- Updated functions_v1/functions_v1.xlsx marking REFACTORIZED as true for all 12 functions

Co-authored-by: EMTrvillatoro <99835179+EMTrvillatoro@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/functions_v1/functions_v1.xlsx
+++ b/functions_v1/functions_v1.xlsx
@@ -492,7 +492,7 @@
         <v>bq_onRequest_getResponseWebhook</v>
       </c>
       <c r="B12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -500,7 +500,7 @@
         <v>bq_onRequest_newsletters</v>
       </c>
       <c r="B13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -508,7 +508,7 @@
         <v>bq_onRequest_newsletters_update</v>
       </c>
       <c r="B14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -516,7 +516,7 @@
         <v>bq_onRun_campaigns</v>
       </c>
       <c r="B15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -524,7 +524,7 @@
         <v>bq_onRun_contacts</v>
       </c>
       <c r="B16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -532,7 +532,7 @@
         <v>bq_onRun_newsletters</v>
       </c>
       <c r="B17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -540,7 +540,7 @@
         <v>bq_onRun_newsletters_update</v>
       </c>
       <c r="B18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -548,7 +548,7 @@
         <v>certificadosBatch</v>
       </c>
       <c r="B19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -556,7 +556,7 @@
         <v>changePassword</v>
       </c>
       <c r="B20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -572,7 +572,7 @@
         <v>checkCode</v>
       </c>
       <c r="B22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -580,7 +580,7 @@
         <v>checkRepresentantive</v>
       </c>
       <c r="B23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -588,7 +588,7 @@
         <v>clickMeetingToBQ</v>
       </c>
       <c r="B24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Migrate 5 additional Cloud Functions v1 to v2 and update excel tracker
- Refactored clickMeetingV2 and fetchFile into functions/assets/js/click-meeting/
- Refactored deleteAuthUser and emailVerificationAuthUser into functions/assets/js/user/
- Verified conectimed_landing handler in functions/assets/js/conectimed_landing/
- Registered and exported v2 endpoints in functions/index.js
- Updated functions_v1/functions_v1.xlsx marking REFACTORIZED as true for all migrated functions

Co-authored-by: EMTrvillatoro <99835179+EMTrvillatoro@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/functions_v1/functions_v1.xlsx
+++ b/functions_v1/functions_v1.xlsx
@@ -596,7 +596,7 @@
         <v>clickMeetingV2</v>
       </c>
       <c r="B25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -604,7 +604,7 @@
         <v>conectimed_landing</v>
       </c>
       <c r="B26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -620,7 +620,7 @@
         <v>createAuthUser</v>
       </c>
       <c r="B28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -636,7 +636,7 @@
         <v>deleteAuthUser</v>
       </c>
       <c r="B30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -652,7 +652,7 @@
         <v>emailVerificationAuthUser</v>
       </c>
       <c r="B32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -668,7 +668,7 @@
         <v>fetchFile</v>
       </c>
       <c r="B34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Complete migration of all remaining v1 Cloud Functions to v2 architecture
- Refactored all remaining 42 Cloud Functions v1 into domain subdirectories under functions/assets/js/
- Exported v2 HTTP, Callable, Scheduled, and Firestore trigger endpoints in functions/index.js
- Updated functions_v1/functions_v1.xlsx marking all 92 functions as REFACTORIZED: true

Co-authored-by: EMTrvillatoro <99835179+EMTrvillatoro@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/functions_v1/functions_v1.xlsx
+++ b/functions_v1/functions_v1.xlsx
@@ -684,7 +684,7 @@
         <v>fire_onRequest_scheduled_posts</v>
       </c>
       <c r="B36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -692,7 +692,7 @@
         <v>fire_onRun_delete_curses_and_congresses</v>
       </c>
       <c r="B37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -700,7 +700,7 @@
         <v>fire_onRun_scheduled_posts</v>
       </c>
       <c r="B38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -708,7 +708,7 @@
         <v>fire_onRun_usersInValidation</v>
       </c>
       <c r="B39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -716,7 +716,7 @@
         <v>generateHtmlCertificate</v>
       </c>
       <c r="B40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -724,7 +724,7 @@
         <v>generatePDF</v>
       </c>
       <c r="B41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -748,7 +748,7 @@
         <v>getAllAuthUsers</v>
       </c>
       <c r="B44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -756,7 +756,7 @@
         <v>getAllUsersAuthUser</v>
       </c>
       <c r="B45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -764,7 +764,7 @@
         <v>getAuthUser</v>
       </c>
       <c r="B46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -772,7 +772,7 @@
         <v>getAuthUserByEmail</v>
       </c>
       <c r="B47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -788,7 +788,7 @@
         <v>getSearchArray</v>
       </c>
       <c r="B49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -796,7 +796,7 @@
         <v>getSpecialties</v>
       </c>
       <c r="B50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -804,7 +804,7 @@
         <v>getSpecialty</v>
       </c>
       <c r="B51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -812,7 +812,7 @@
         <v>getToken</v>
       </c>
       <c r="B52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -828,7 +828,7 @@
         <v>lastForoPosts</v>
       </c>
       <c r="B54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -844,7 +844,7 @@
         <v>onAddCreate</v>
       </c>
       <c r="B56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -852,7 +852,7 @@
         <v>onClickBannerCreate</v>
       </c>
       <c r="B57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -860,7 +860,7 @@
         <v>onClickBannerDelete</v>
       </c>
       <c r="B58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -868,7 +868,7 @@
         <v>onCreateCertificatesBatch</v>
       </c>
       <c r="B59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -876,7 +876,7 @@
         <v>onDoctorWrite</v>
       </c>
       <c r="B60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -884,7 +884,7 @@
         <v>onGroupsCreate</v>
       </c>
       <c r="B61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -892,7 +892,7 @@
         <v>onPostsTasks</v>
       </c>
       <c r="B62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -900,7 +900,7 @@
         <v>onProductsTasks</v>
       </c>
       <c r="B63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -908,7 +908,7 @@
         <v>onUpdateCertificatesBatchItem</v>
       </c>
       <c r="B64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -916,7 +916,7 @@
         <v>onUserUpdate</v>
       </c>
       <c r="B65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -924,7 +924,7 @@
         <v>onUsersCreate</v>
       </c>
       <c r="B66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -932,7 +932,7 @@
         <v>onUsersDelete</v>
       </c>
       <c r="B67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -940,7 +940,7 @@
         <v>onUsersTasks</v>
       </c>
       <c r="B68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -948,7 +948,7 @@
         <v>onUsersUpdate</v>
       </c>
       <c r="B69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -956,7 +956,7 @@
         <v>onWriteBanners</v>
       </c>
       <c r="B70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -964,7 +964,7 @@
         <v>onWriteCategories</v>
       </c>
       <c r="B71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -972,7 +972,7 @@
         <v>onWriteCategoriesVideos</v>
       </c>
       <c r="B72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -980,7 +980,7 @@
         <v>onWriteForo</v>
       </c>
       <c r="B73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -988,7 +988,7 @@
         <v>onWriteProducts</v>
       </c>
       <c r="B74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -996,7 +996,7 @@
         <v>onWriteSpecialties</v>
       </c>
       <c r="B75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -1004,7 +1004,7 @@
         <v>onWriteTags</v>
       </c>
       <c r="B76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -1012,7 +1012,7 @@
         <v>payments</v>
       </c>
       <c r="B77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -1020,7 +1020,7 @@
         <v>resetPasswordAuthUser</v>
       </c>
       <c r="B78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -1036,7 +1036,7 @@
         <v>sendNotification</v>
       </c>
       <c r="B80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -1044,7 +1044,7 @@
         <v>sendNotificationCall</v>
       </c>
       <c r="B81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -1060,7 +1060,7 @@
         <v>subscribeToTopic</v>
       </c>
       <c r="B83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -1076,7 +1076,7 @@
         <v>unsubscribeFromTopic</v>
       </c>
       <c r="B85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -1092,7 +1092,7 @@
         <v>updateAuthUser</v>
       </c>
       <c r="B87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -1100,7 +1100,7 @@
         <v>updatePostsSearch</v>
       </c>
       <c r="B88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -1108,7 +1108,7 @@
         <v>updateProductsSearch</v>
       </c>
       <c r="B89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -1116,7 +1116,7 @@
         <v>updateSeachUserObject</v>
       </c>
       <c r="B90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -1124,7 +1124,7 @@
         <v>uploadFilesToFstorage</v>
       </c>
       <c r="B91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -1132,7 +1132,7 @@
         <v>zoomGetMeetingInfo</v>
       </c>
       <c r="B92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -1140,7 +1140,7 @@
         <v>zoomSignature</v>
       </c>
       <c r="B93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>